<commit_message>
PAUSED (task182, task192, task195): checkpoint, three passes mid-pass
Continues 5d158e5. task182 and task192 are writing up their notes, task192's against the
rulings on its four open calls, and task195 is on the pre-ship realism pass: the
read-set identifier strides, two uniform measurement columns, the typed-marker count,
the automatic calls that sit exactly at their threshold, and the three document date
contradictions.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task195/golden/screen_change_validation_2027q3.xlsx
+++ b/task195/golden/screen_change_validation_2027q3.xlsx
@@ -1380,10 +1380,10 @@
         <v>9</v>
       </c>
       <c r="D4" s="17">
-        <v>0.878</v>
+        <v>1</v>
       </c>
       <c r="E4" s="7">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>